<commit_message>
news: three awards 2026 as lead story; fix Paffenbarger interval; Hokkaido page to past tense; update news checker
</commit_message>
<xml_diff>
--- a/news/news-checker.xlsx
+++ b/news/news-checker.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTA(D7:D47)</f>
+        <f>COUNTA(D7:D50)</f>
         <v/>
       </c>
       <c r="C5" t="inlineStr">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="D5">
-        <f>COUNTIF(J7:J47,"Done")</f>
+        <f>COUNTIF(J7:J50,"Done")</f>
         <v/>
       </c>
       <c r="E5" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="F5">
-        <f>COUNTIF(J7:J47,"Asset ready")</f>
+        <f>COUNTIF(J7:J50,"Asset ready")</f>
         <v/>
       </c>
       <c r="G5" t="inlineStr">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="H5">
-        <f>COUNTIF(J7:J47,"To do")</f>
+        <f>COUNTIF(J7:J50,"To do")</f>
         <v/>
       </c>
     </row>
@@ -593,17 +593,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>October 2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists 2026</t>
+          <t>Three awards recognise a shared vision for the dental materials that should exist</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2026</t>
+          <t>three-awards-2026</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2026.html</t>
+          <t>news/three-awards-2026.html</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>top2pct-2026.png</t>
+          <t>three-awards-2026-hero.jpg</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>EN/ES/PT/FR/中文</t>
+          <t>EN/ES/PT/FR/中文/AR</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Latest edition (6th)</t>
+          <t>Lead story on news.html (lead:true). Combines IADR Innovation 2026, IADR-SEA Hatton Senior 2026 and ADM Paffenbarger 2026</t>
         </is>
       </c>
     </row>
@@ -643,22 +643,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>9 October 2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of the Journal of Clinical Periodontology</t>
+          <t>Clarice Sabino Receives the Academy of Dental Materials Paffenbarger Award</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>jcp-editorial-board-2026</t>
+          <t>adm-paffenbarger-award-clarice-sabino-2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>news/jcp-editorial-board-2026.html</t>
+          <t>news/adm-paffenbarger-award-clarice-sabino-2026.html</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -678,12 +678,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>EN/ES/PT/FR/中文</t>
+          <t>EN/ES/PT/FR/中文/AR</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Supervisor: A/P Rosa. Interval corrected to three weeks after the Hatton (2026-10-15)</t>
         </is>
       </c>
     </row>
@@ -698,17 +703,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>June 2026</t>
+          <t>September 2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A/P Rosa's guidance article on biocompatibility highlighted in Dental Materials (JCR 2025)</t>
+          <t>Clarice Sabino Receives the IADR Hatton Award SEA in the Senior Category</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>biocompatibility-guidance-jcr-dental-materials-2025</t>
+          <t>iadr-sea-hatton-senior-clarice-sabino-2026</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -718,17 +723,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>news/biocompatibility-guidance-jcr-dental-materials-2025.html</t>
+          <t>news/iadr-sea-hatton-senior-clarice-sabino-2026.html</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>biocompatibility-guidance-jcr-2025.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>EN/ES/PT/FR/中文</t>
+          <t>EN/ES/PT/FR/中文/AR</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -738,7 +743,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>JCR 2025 — 5th most cited contributor; 29 citations</t>
+          <t>Supervisor: A/P Rosa. IADR-SEA 2026, Phnom Penh, 17–19 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -748,22 +753,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Press</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>May 2026</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The Straits Times features A/P Rosa's AI-enabled living laboratory models</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists 2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>straits-times-ai-models</t>
+          <t>top2pct-scientists-2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -773,12 +778,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>news/straits-times-ai-models.html</t>
+          <t>news/top2pct-scientists-2026.html</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>straits-times-ai-models.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -793,7 +798,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Image updated — Living Lab.png (941×1672, cropped 16:9)</t>
+          <t>Latest edition (6th); hero file missing from disk, page fixed to no-photo 2026-08-04, needs new hero</t>
         </is>
       </c>
     </row>
@@ -803,22 +808,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>March 2026</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A/P Rosa receives the 2026 IADR Innovation in Oral Care Award</t>
+          <t>A/P Rosa joins the Editorial Board of the Journal of Clinical Periodontology</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>iadr-innovation-award-2026</t>
+          <t>jcp-editorial-board-2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -828,12 +833,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>news/iadr-innovation-award-2026.html</t>
+          <t>news/jcp-editorial-board-2026.html</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>iadr-ceremony.jpg</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -844,11 +849,6 @@
       <c r="J11" s="4" t="inlineStr">
         <is>
           <t>Done</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Photo 4:3; CTAs link to iadr.org</t>
         </is>
       </c>
     </row>
@@ -858,22 +858,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>February 2026</t>
+          <t>June 2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed to Singapore's National Mirror Working Group for ISO/TC 194</t>
+          <t>A/P Rosa's guidance article on biocompatibility highlighted in Dental Materials (JCR 2025)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>iso-tc194-mirror-group</t>
+          <t>biocompatibility-guidance-jcr-dental-materials-2025</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -883,12 +883,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>news/iso-tc194-mirror-group.html</t>
+          <t>news/biocompatibility-guidance-jcr-dental-materials-2025.html</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>biocompatibility-guidance-jcr-2025.png</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>CTA placeholders (#)</t>
+          <t>JCR 2025 — 5th most cited contributor; 29 citations</t>
         </is>
       </c>
     </row>
@@ -913,22 +913,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Press</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>September 2025</t>
+          <t>May 2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists 2025 (5th year)</t>
+          <t>The Straits Times features A/P Rosa's AI-enabled living laboratory models</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2025</t>
+          <t>straits-times-ai-models</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -938,12 +938,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2025.html</t>
+          <t>news/straits-times-ai-models.html</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>top2pct-2025.png</t>
+          <t>straits-times-ai-models.png</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>5th year; ranked top 1.3%</t>
+          <t>Image updated — Living Lab.png (941×1672, cropped 16:9)</t>
         </is>
       </c>
     </row>
@@ -968,22 +968,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>August 2025</t>
+          <t>March 2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>The science behind toothpaste</t>
+          <t>A/P Rosa receives the 2026 IADR Innovation in Oral Care Award</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>science-behind-toothpaste-2025</t>
+          <t>iadr-innovation-award-2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -993,12 +993,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>news/science-behind-toothpaste-2025.html</t>
+          <t>news/iadr-innovation-award-2026.html</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>science-behind-toothpaste-2025.png</t>
+          <t>iadr-ceremony.jpg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1006,14 +1006,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>Photo 4:3; CTAs link to iadr.org</t>
         </is>
       </c>
     </row>
@@ -1023,22 +1023,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>April 2025</t>
+          <t>February 2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Accelerating biomaterials development with neural-network strategies</t>
+          <t>A/P Rosa appointed to Singapore's National Mirror Working Group for ISO/TC 194</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>neural-networks-biomaterials-2025</t>
+          <t>iso-tc194-mirror-group</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>news/neural-networks-biomaterials-2025.html</t>
+          <t>news/iso-tc194-mirror-group.html</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>neural-networks-biomaterials-2025.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1061,14 +1061,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>CTA placeholders (#)</t>
         </is>
       </c>
     </row>
@@ -1078,22 +1078,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>September 2025</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the inaugural Meet the Fellows session (Academy of Dental Materials)</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists 2025 (5th year)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>adm-meet-the-fellows-2025</t>
+          <t>top2pct-scientists-2025</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1103,12 +1103,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>news/adm-meet-the-fellows-2025.html</t>
+          <t>news/top2pct-scientists-2025.html</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>adm-meet-the-fellows.png</t>
+          <t>top2pct-2025.png</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Category set to Institutional in news.js</t>
+          <t>5th year; ranked top 1.3%</t>
         </is>
       </c>
     </row>
@@ -1133,22 +1133,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>August 2025</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the editorial board of the European Journal of Oral Sciences</t>
+          <t>The science behind toothpaste</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ejos-editorial-board-2024</t>
+          <t>science-behind-toothpaste-2025</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1158,12 +1158,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>news/ejos-editorial-board-2024.html</t>
+          <t>news/science-behind-toothpaste-2025.html</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>science-behind-toothpaste-2025.png</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1171,9 +1171,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -1183,22 +1188,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>April 2025</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of Discover Nano</t>
+          <t>Accelerating biomaterials development with neural-network strategies</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>discover-nano-editorial-board-2024</t>
+          <t>neural-networks-biomaterials-2025</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1208,12 +1213,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>news/discover-nano-editorial-board-2024.html</t>
+          <t>news/neural-networks-biomaterials-2025.html</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>neural-networks-biomaterials-2025.png</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1221,9 +1226,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -1233,22 +1243,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>March 2025</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists 2024</t>
+          <t>A/P Rosa joins the inaugural Meet the Fellows session (Academy of Dental Materials)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2024</t>
+          <t>adm-meet-the-fellows-2025</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1258,12 +1268,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2024.html</t>
+          <t>news/adm-meet-the-fellows-2025.html</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>top2pct-2024.png</t>
+          <t>adm-meet-the-fellows.png</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1278,7 +1288,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4th consecutive year</t>
+          <t>Category set to Institutional in news.js</t>
         </is>
       </c>
     </row>
@@ -1288,22 +1298,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>December 2024</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A/P Rosa co-authors guidance on biocompatibility and dental-pulp regeneration</t>
+          <t>A/P Rosa joins the editorial board of the European Journal of Oral Sciences</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>guidance-biocompat-pulp-2024</t>
+          <t>ejos-editorial-board-2024</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1313,7 +1323,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>news/guidance-biocompat-pulp-2024.html</t>
+          <t>news/ejos-editorial-board-2024.html</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1326,14 +1336,9 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>No hero image</t>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1353,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>October 2024</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed to the Board of Directors of the Academy of Dental Materials</t>
+          <t>A/P Rosa joins the Editorial Board of Discover Nano</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>adm-board-member-2024</t>
+          <t>discover-nano-editorial-board-2024</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1368,12 +1373,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>news/adm-board-member-2024.html</t>
+          <t>news/discover-nano-editorial-board-2024.html</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>adm-board.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1384,11 +1389,6 @@
       <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Done</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>CTA placeholder (#)</t>
         </is>
       </c>
     </row>
@@ -1398,22 +1398,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 2024</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Berita Harian features the NUCOHS Tooth Tissue Bank</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists 2024</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>berita-harian-tooth-bank-2024</t>
+          <t>top2pct-scientists-2024</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1423,12 +1423,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>news/berita-harian-tooth-bank-2024.html</t>
+          <t>news/top2pct-scientists-2024.html</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>berita-harian-tooth-bank-2024.webp</t>
+          <t>top2pct-2024.png</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1436,14 +1436,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>4th consecutive year</t>
         </is>
       </c>
     </row>
@@ -1458,17 +1458,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>August 2024</t>
+          <t>December 2024</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Channel NewsAsia interviews A/P Rosa on the Tooth Tissue Bank</t>
+          <t>A/P Rosa co-authors guidance on biocompatibility and dental-pulp regeneration</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>cna-tooth-bank-2024</t>
+          <t>guidance-biocompat-pulp-2024</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>news/cna-tooth-bank-2024.html</t>
+          <t>news/guidance-biocompat-pulp-2024.html</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>cna-tooth-bank-2024.jpg</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>No hero image</t>
         </is>
       </c>
     </row>
@@ -1508,22 +1508,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Press</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>July 2024</t>
+          <t>October 2024</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>The Straits Times: how Singapore's first Tooth Tissue Bank is advancing dental research</t>
+          <t>A/P Rosa appointed to the Board of Directors of the Academy of Dental Materials</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>straits-times-tooth-bank-2024</t>
+          <t>adm-board-member-2024</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>news/straits-times-tooth-bank-2024.html</t>
+          <t>news/adm-board-member-2024.html</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>adm-board.png</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>ST article screenshot (tooth-bank-st.png)</t>
+          <t>CTA placeholder (#)</t>
         </is>
       </c>
     </row>
@@ -1563,22 +1563,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>March 2024</t>
+          <t>September 2024</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A/P Rosa concludes his term as president of the IADR Dental Materials Group</t>
+          <t>Berita Harian features the NUCOHS Tooth Tissue Bank</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>iadr-dmg-president-end-2024</t>
+          <t>berita-harian-tooth-bank-2024</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1588,12 +1588,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>news/iadr-dmg-president-end-2024.html</t>
+          <t>news/berita-harian-tooth-bank-2024.html</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>iadr-dmg-president-2024.png</t>
+          <t>berita-harian-tooth-bank-2024.webp</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1618,22 +1618,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>August 2024</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Clarice Sabino wins the 2023 IADR Kulzer Travel Award</t>
+          <t>Channel NewsAsia interviews A/P Rosa on the Tooth Tissue Bank</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>iadr-kulzer-travel-award-clarice-sabino-2023</t>
+          <t>cna-tooth-bank-2024</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>news/iadr-kulzer-travel-award-clarice-sabino-2023.html</t>
+          <t>news/cna-tooth-bank-2024.html</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>iadr-kulzer-award-clarice-sabino-2023.jpg</t>
+          <t>cna-tooth-bank-2024.jpg</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1656,9 +1656,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -1668,22 +1673,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Press</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Priti Pragati Rath receives the IADR Kulzer Award 2023</t>
+          <t>The Straits Times: how Singapore's first Tooth Tissue Bank is advancing dental research</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>iadr-kulzer-award-priti-pragati-rath-2023</t>
+          <t>straits-times-tooth-bank-2024</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1693,12 +1698,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>news/iadr-kulzer-award-priti-pragati-rath-2023.html</t>
+          <t>news/straits-times-tooth-bank-2024.html</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>iadr-kulzer-award-priti-pragati-rath.jpg</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1713,7 +1718,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Supervisor: A/P Rosa</t>
+          <t>ST article screenshot (tooth-bank-st.png)</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1728,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>November 2023</t>
+          <t>March 2024</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>A/P Rosa's work selected for the JDR Editor's Choice Collection 2023</t>
+          <t>A/P Rosa concludes his term as president of the IADR Dental Materials Group</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>jdr-editors-choice-collection-2023</t>
+          <t>iadr-dmg-president-end-2024</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1748,12 +1753,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>news/jdr-editors-choice-collection-2023.html</t>
+          <t>news/iadr-dmg-president-end-2024.html</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>jdr-editor-choice-2023.png</t>
+          <t>iadr-dmg-president-2024.png</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1761,9 +1766,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -1778,17 +1788,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>October 2023</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A/P Rosa becomes a Fellow of the Academy of Dental Materials</t>
+          <t>Clarice Sabino wins the 2023 IADR Kulzer Travel Award</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>adm-fellow-2023</t>
+          <t>iadr-kulzer-travel-award-clarice-sabino-2023</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1798,12 +1808,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>news/adm-fellow-2023.html</t>
+          <t>news/iadr-kulzer-travel-award-clarice-sabino-2023.html</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>iadr-kulzer-award-clarice-sabino-2023.jpg</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1811,14 +1821,9 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>No hero image</t>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1833,17 +1838,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>October 2023</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A/P Rosa recognised in the World's Top 2% most-cited scientists 2023</t>
+          <t>Priti Pragati Rath receives the IADR Kulzer Award 2023</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2023</t>
+          <t>iadr-kulzer-award-priti-pragati-rath-2023</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1853,12 +1858,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2023.html</t>
+          <t>news/iadr-kulzer-award-priti-pragati-rath-2023.html</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>top2pct-2023.png</t>
+          <t>iadr-kulzer-award-priti-pragati-rath.jpg</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1873,7 +1878,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>3rd consecutive year</t>
+          <t>Supervisor: A/P Rosa</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1893,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>April 2023</t>
+          <t>November 2023</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>UFPEL and NUS win One Health research grants</t>
+          <t>A/P Rosa's work selected for the JDR Editor's Choice Collection 2023</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ufpel-nus-one-health-2023</t>
+          <t>jdr-editors-choice-collection-2023</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1908,12 +1913,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>news/ufpel-nus-one-health-2023.html</t>
+          <t>news/jdr-editors-choice-collection-2023.html</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>ufpel-nus-research-collaboration.png</t>
+          <t>jdr-editor-choice-2023.png</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1921,14 +1926,9 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Needs asset; text in PDFs</t>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1943,17 +1943,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>October 2022</t>
+          <t>October 2023</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists (2nd consecutive year)</t>
+          <t>A/P Rosa becomes a Fellow of the Academy of Dental Materials</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2022</t>
+          <t>adm-fellow-2023</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1963,12 +1963,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2022.html</t>
+          <t>news/adm-fellow-2023.html</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>top2pct-2022.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1976,14 +1976,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J32" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2nd consecutive year</t>
+          <t>No hero image</t>
         </is>
       </c>
     </row>
@@ -1998,17 +1998,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>October 2023</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Melissa Koh receives the IADR Pediatric Oral Health Research Group Student Award 2021</t>
+          <t>A/P Rosa recognised in the World's Top 2% most-cited scientists 2023</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>iadr-pediatric-award-melissa-koh-2021</t>
+          <t>top2pct-scientists-2023</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2018,12 +2018,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>news/iadr-pediatric-award-melissa-koh-2021.html</t>
+          <t>news/top2pct-scientists-2023.html</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>top2pct-2023.png</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Supervisor: A/P Rosa</t>
+          <t>3rd consecutive year</t>
         </is>
       </c>
     </row>
@@ -2053,17 +2053,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>July 2021</t>
+          <t>April 2023</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>A/P Rosa receives the 2021 IADR Stephen Bayne Mid-Career Award</t>
+          <t>UFPEL and NUS win One Health research grants</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>iadr-bayne-midcareer-2021</t>
+          <t>ufpel-nus-one-health-2023</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2073,12 +2073,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>news/iadr-bayne-midcareer-award-2021.html</t>
+          <t>news/ufpel-nus-one-health-2023.html</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>iadr-bayne-midcareer-award-2021.jpg</t>
+          <t>ufpel-nus-research-collaboration.png</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2108,17 +2108,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>July 2021</t>
+          <t>October 2022</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A/P Rosa receives the IADR Distinguished Young Investigator Award</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists (2nd consecutive year)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>iadr-young-investigator-2021</t>
+          <t>top2pct-scientists-2022</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2128,12 +2128,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>news/iadr-young-investigator-award-2021.html</t>
+          <t>news/top2pct-scientists-2022.html</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>iadr-young-investigator-award-2021.webp</t>
+          <t>top2pct-2022.png</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2141,14 +2141,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J35" s="6" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>2nd consecutive year</t>
         </is>
       </c>
     </row>
@@ -2163,17 +2163,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>July 2021</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Four NUS Dentistry researchers in the World's Top 2% most-cited scientists</t>
+          <t>Melissa Koh receives the IADR Pediatric Oral Health Research Group Student Award 2021</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2021</t>
+          <t>iadr-pediatric-award-melissa-koh-2021</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2021.html</t>
+          <t>news/iadr-pediatric-award-melissa-koh-2021.html</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>top2pct-2021.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>One of four NUS Dentistry researchers that year</t>
+          <t>Supervisor: A/P Rosa</t>
         </is>
       </c>
     </row>
@@ -2218,17 +2218,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>June 2021</t>
+          <t>July 2021</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Best graphical abstract — eCells &amp; Materials</t>
+          <t>A/P Rosa receives the 2021 IADR Stephen Bayne Mid-Career Award</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ecm-graphical-abstract-2021</t>
+          <t>iadr-bayne-midcareer-2021</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2238,12 +2238,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>news/ecm-graphical-abstract-2021.html</t>
+          <t>news/iadr-bayne-midcareer-award-2021.html</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>ecm-graphical-abstract-2021.jpg</t>
+          <t>iadr-bayne-midcareer-award-2021.jpg</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Ultra-wide 858×229; contain mode</t>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -2268,22 +2268,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>July 2021</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of Dental Materials</t>
+          <t>A/P Rosa receives the IADR Distinguished Young Investigator Award</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>dental-materials-editorial-board-2020</t>
+          <t>iadr-young-investigator-2021</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2293,12 +2293,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>news/dental-materials-editorial-board-2020.html</t>
+          <t>news/iadr-young-investigator-award-2021.html</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>iadr-young-investigator-award-2021.webp</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2306,9 +2306,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -2318,22 +2323,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>July 2021</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of JADA FS</t>
+          <t>Four NUS Dentistry researchers in the World's Top 2% most-cited scientists</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>jada-fs-editorial-board-2020</t>
+          <t>top2pct-scientists-2021</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2343,12 +2348,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>news/jada-fs-editorial-board-2020.html</t>
+          <t>news/top2pct-scientists-2021.html</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>top2pct-2021.png</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2359,6 +2364,11 @@
       <c r="J39" s="4" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>One of four NUS Dentistry researchers that year</t>
         </is>
       </c>
     </row>
@@ -2368,22 +2378,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>June 2021</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed Associate Editor of the Journal of Prosthodontics</t>
+          <t>Best graphical abstract — eCells &amp; Materials</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>journal-prosthodontics-associate-editor-2020</t>
+          <t>ecm-graphical-abstract-2021</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2393,12 +2403,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>news/journal-prosthodontics-associate-editor-2020.html</t>
+          <t>news/ecm-graphical-abstract-2021.html</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ecm-graphical-abstract-2021.jpg</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2406,9 +2416,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Ultra-wide 858×229; contain mode</t>
         </is>
       </c>
     </row>
@@ -2418,22 +2433,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Institutional</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>December 2020</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Dental DART — protective tent for safer dentistry during the pandemic</t>
+          <t>A/P Rosa joins the Editorial Board of Dental Materials</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>dental-dart-aerosol-2020</t>
+          <t>dental-materials-editorial-board-2020</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2443,12 +2458,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>news/dental-dart-aerosol-2020.html</t>
+          <t>news/dental-materials-editorial-board-2020.html</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>dental-dart-01…04.jpg</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2463,7 +2478,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>COVID-era aerosol shield; 4 photos</t>
+          <t>No hero image (had a mismatched RSC Sustainability cover wired in by mistake, removed 2026-08-04)</t>
         </is>
       </c>
     </row>
@@ -2473,22 +2488,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>February 2020</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Two papers among the 25 most-cited in Dental Materials</t>
+          <t>A/P Rosa joins the Editorial Board of JADA FS</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>dental-materials-top25-2020</t>
+          <t>jada-fs-editorial-board-2020</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2498,12 +2513,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>news/dental-materials-top25-2020.html</t>
+          <t>news/jada-fs-editorial-board-2020.html</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>dental-materials-top25-2020.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2511,14 +2526,9 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Needs asset; text in PDFs</t>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2533,17 +2543,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Scientific Advisory Board of the Journal of Endodontics</t>
+          <t>A/P Rosa appointed Associate Editor of the Journal of Prosthodontics</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>joe-scientific-advisory-board-2019</t>
+          <t>journal-prosthodontics-associate-editor-2020</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2553,7 +2563,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>news/joe-scientific-advisory-board-2019.html</t>
+          <t>news/journal-prosthodontics-associate-editor-2020.html</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2578,22 +2588,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Institutional</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>December 2020</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed Associate Editor of Emergent Materials</t>
+          <t>Dental DART — protective tent for safer dentistry during the pandemic</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>emergent-materials-associate-editor-2019</t>
+          <t>dental-dart-aerosol-2020</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2603,12 +2613,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>news/emergent-materials-associate-editor-2019.html</t>
+          <t>news/dental-dart-aerosol-2020.html</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>dental-dart-01…04.jpg</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2619,6 +2629,11 @@
       <c r="J44" s="4" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>COVID-era aerosol shield; 4 photos</t>
         </is>
       </c>
     </row>
@@ -2633,17 +2648,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>February 2020</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Klara Koh receives the IADR-SEA Hatton Award Junior Category 2018</t>
+          <t>Two papers among the 25 most-cited in Dental Materials</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>iadr-sea-hatton-junior-klara-koh-2018</t>
+          <t>dental-materials-top25-2020</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2653,12 +2668,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>news/iadr-sea-hatton-junior-klara-koh-2018.html</t>
+          <t>news/dental-materials-top25-2020.html</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>dental-materials-top25-2020.png</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2666,14 +2681,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J45" s="4" t="inlineStr">
+      <c r="J45" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Supervisor: A/P Rosa</t>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -2688,17 +2703,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of the Journal of Dental Research</t>
+          <t>A/P Rosa joins the Scientific Advisory Board of the Journal of Endodontics</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>jdr-editorial-board-2018</t>
+          <t>joe-scientific-advisory-board-2019</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2708,7 +2723,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>news/jdr-editorial-board-2018.html</t>
+          <t>news/joe-scientific-advisory-board-2019.html</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2733,50 +2748,210 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>Appointment</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>A/P Rosa appointed Associate Editor of Emergent Materials</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>emergent-materials-associate-editor-2019</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>news/emergent-materials-associate-editor-2019.html</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>EN/ES/PT/FR/中文</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>42</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>Award</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Klara Koh receives the IADR-SEA Hatton Award Junior Category 2018</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>iadr-sea-hatton-junior-klara-koh-2018</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>news/iadr-sea-hatton-junior-klara-koh-2018.html</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>EN/ES/PT/FR/中文</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Supervisor: A/P Rosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>43</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Appointment</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>A/P Rosa joins the Editorial Board of the Journal of Dental Research</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>jdr-editorial-board-2018</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>news/jdr-editorial-board-2018.html</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>EN/ES/PT/FR/中文</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>No hero image (had the jdr-editors-choice-collection-2023 paper card wired in by mistake, removed 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>44</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Award</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
         <is>
           <t>November 2018</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Two of A/P Rosa's papers among the 100 most-cited in regenerative endodontics</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>two-top-cited-papers-regenerative-endodontics-2018</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
         <is>
           <t>news/two-top-cited-papers-regenerative-endodontics-2018.html</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>two-top-cited-regenerative-endodontics.png</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>EN/ES/PT/FR/中文</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>EN/ES/PT/FR/中文</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t>#26 JDR 2013 / #98 Int Dent J 2011 per JOE 2018 bibliometric analysis</t>
         </is>

</xml_diff>

<commit_message>
news: Straits Times Dyson collaboration; three awards lead story; Hokkaido past tense; who trainee award; news checker
</commit_message>
<xml_diff>
--- a/news/news-checker.xlsx
+++ b/news/news-checker.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -495,7 +494,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTA(D7:D50)</f>
+        <f>COUNTA(D7:D51)</f>
         <v/>
       </c>
       <c r="C5" t="inlineStr">
@@ -504,7 +503,7 @@
         </is>
       </c>
       <c r="D5">
-        <f>COUNTIF(J7:J50,"Done")</f>
+        <f>COUNTIF(J7:J51,"Done")</f>
         <v/>
       </c>
       <c r="E5" t="inlineStr">
@@ -513,7 +512,7 @@
         </is>
       </c>
       <c r="F5">
-        <f>COUNTIF(J7:J50,"Asset ready")</f>
+        <f>COUNTIF(J7:J51,"Asset ready")</f>
         <v/>
       </c>
       <c r="G5" t="inlineStr">
@@ -522,7 +521,7 @@
         </is>
       </c>
       <c r="H5">
-        <f>COUNTIF(J7:J50,"To do")</f>
+        <f>COUNTIF(J7:J51,"To do")</f>
         <v/>
       </c>
     </row>
@@ -754,22 +753,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Media Feature</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>10 September 2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists 2026</t>
+          <t>The Straits Times highlights A/P Rosa's research collaboration with Dyson</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2026</t>
+          <t>straits-times-dyson-2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -779,7 +778,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2026.html</t>
+          <t>news/straits-times-dyson-2026.html</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -789,7 +788,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>EN/ES/PT/FR/中文</t>
+          <t>EN/ES/PT/FR/中文/AR</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -799,7 +798,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Latest edition (6th); hero file missing from disk, page fixed to no-photo 2026-08-04, needs new hero</t>
+          <t>No hero image. Source: The Straits Times, 10 Sep 2026 (Yamini Chinnuswamy)</t>
         </is>
       </c>
     </row>
@@ -809,7 +808,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -819,12 +818,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of the Journal of Clinical Periodontology</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists 2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>jcp-editorial-board-2026</t>
+          <t>top2pct-scientists-2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -834,7 +833,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>news/jcp-editorial-board-2026.html</t>
+          <t>news/top2pct-scientists-2026.html</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -850,6 +849,11 @@
       <c r="J11" s="4" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Latest edition (6th); hero file missing from disk, page fixed to no-photo 2026-08-04, needs new hero</t>
         </is>
       </c>
     </row>
@@ -859,22 +863,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>June 2026</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>A/P Rosa's guidance article on biocompatibility highlighted in Dental Materials (JCR 2025)</t>
+          <t>A/P Rosa joins the Editorial Board of the Journal of Clinical Periodontology</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>biocompatibility-guidance-jcr-dental-materials-2025</t>
+          <t>jcp-editorial-board-2026</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -884,12 +888,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>news/biocompatibility-guidance-jcr-dental-materials-2025.html</t>
+          <t>news/jcp-editorial-board-2026.html</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>biocompatibility-guidance-jcr-2025.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -900,11 +904,6 @@
       <c r="J12" s="4" t="inlineStr">
         <is>
           <t>Done</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>JCR 2025 — 5th most cited contributor; 29 citations</t>
         </is>
       </c>
     </row>
@@ -914,22 +913,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Press</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>May 2026</t>
+          <t>June 2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The Straits Times features A/P Rosa's AI-enabled living laboratory models</t>
+          <t>A/P Rosa's guidance article on biocompatibility highlighted in Dental Materials (JCR 2025)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>straits-times-ai-models</t>
+          <t>biocompatibility-guidance-jcr-dental-materials-2025</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -939,12 +938,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>news/straits-times-ai-models.html</t>
+          <t>news/biocompatibility-guidance-jcr-dental-materials-2025.html</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>straits-times-ai-models.png</t>
+          <t>biocompatibility-guidance-jcr-2025.png</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -959,7 +958,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Image updated — Living Lab.png (941×1672, cropped 16:9)</t>
+          <t>JCR 2025 — 5th most cited contributor; 29 citations</t>
         </is>
       </c>
     </row>
@@ -969,22 +968,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Press</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>March 2026</t>
+          <t>May 2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A/P Rosa receives the 2026 IADR Innovation in Oral Care Award</t>
+          <t>The Straits Times features A/P Rosa's AI-enabled living laboratory models</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>iadr-innovation-award-2026</t>
+          <t>straits-times-ai-models</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -994,12 +993,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>news/iadr-innovation-award-2026.html</t>
+          <t>news/straits-times-ai-models.html</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>iadr-ceremony.jpg</t>
+          <t>straits-times-ai-models.png</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1014,7 +1013,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Photo 4:3; CTAs link to iadr.org</t>
+          <t>Image updated — Living Lab.png (941×1672, cropped 16:9)</t>
         </is>
       </c>
     </row>
@@ -1024,22 +1023,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>February 2026</t>
+          <t>March 2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed to Singapore's National Mirror Working Group for ISO/TC 194</t>
+          <t>A/P Rosa receives the 2026 IADR Innovation in Oral Care Award</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>iso-tc194-mirror-group</t>
+          <t>iadr-innovation-award-2026</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1049,12 +1048,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>news/iso-tc194-mirror-group.html</t>
+          <t>news/iadr-innovation-award-2026.html</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>iadr-ceremony.jpg</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1069,7 +1068,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>CTA placeholders (#)</t>
+          <t>Photo 4:3; CTAs link to iadr.org</t>
         </is>
       </c>
     </row>
@@ -1079,22 +1078,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>September 2025</t>
+          <t>February 2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists 2025 (5th year)</t>
+          <t>A/P Rosa appointed to Singapore's National Mirror Working Group for ISO/TC 194</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2025</t>
+          <t>iso-tc194-mirror-group</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1104,12 +1103,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2025.html</t>
+          <t>news/iso-tc194-mirror-group.html</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>top2pct-2025.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1124,7 +1123,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>5th year; ranked top 1.3%</t>
+          <t>CTA placeholders (#)</t>
         </is>
       </c>
     </row>
@@ -1134,22 +1133,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>August 2025</t>
+          <t>September 2025</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>The science behind toothpaste</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists 2025 (5th year)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>science-behind-toothpaste-2025</t>
+          <t>top2pct-scientists-2025</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1159,12 +1158,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>news/science-behind-toothpaste-2025.html</t>
+          <t>news/top2pct-scientists-2025.html</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>science-behind-toothpaste-2025.png</t>
+          <t>top2pct-2025.png</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1172,14 +1171,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>5th year; ranked top 1.3%</t>
         </is>
       </c>
     </row>
@@ -1194,17 +1193,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>April 2025</t>
+          <t>August 2025</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Accelerating biomaterials development with neural-network strategies</t>
+          <t>The science behind toothpaste</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>neural-networks-biomaterials-2025</t>
+          <t>science-behind-toothpaste-2025</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1214,12 +1213,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>news/neural-networks-biomaterials-2025.html</t>
+          <t>news/science-behind-toothpaste-2025.html</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>neural-networks-biomaterials-2025.png</t>
+          <t>science-behind-toothpaste-2025.png</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1249,17 +1248,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>April 2025</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the inaugural Meet the Fellows session (Academy of Dental Materials)</t>
+          <t>Accelerating biomaterials development with neural-network strategies</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>adm-meet-the-fellows-2025</t>
+          <t>neural-networks-biomaterials-2025</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1269,12 +1268,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>news/adm-meet-the-fellows-2025.html</t>
+          <t>news/neural-networks-biomaterials-2025.html</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>adm-meet-the-fellows.png</t>
+          <t>neural-networks-biomaterials-2025.png</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1282,14 +1281,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Category set to Institutional in news.js</t>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -1299,22 +1298,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>March 2025</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the editorial board of the European Journal of Oral Sciences</t>
+          <t>A/P Rosa joins the inaugural Meet the Fellows session (Academy of Dental Materials)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ejos-editorial-board-2024</t>
+          <t>adm-meet-the-fellows-2025</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1324,12 +1323,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>news/ejos-editorial-board-2024.html</t>
+          <t>news/adm-meet-the-fellows-2025.html</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>adm-meet-the-fellows.png</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1340,6 +1339,11 @@
       <c r="J20" s="4" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Category set to Institutional in news.js</t>
         </is>
       </c>
     </row>
@@ -1359,12 +1363,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of Discover Nano</t>
+          <t>A/P Rosa joins the editorial board of the European Journal of Oral Sciences</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>discover-nano-editorial-board-2024</t>
+          <t>ejos-editorial-board-2024</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1374,7 +1378,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>news/discover-nano-editorial-board-2024.html</t>
+          <t>news/ejos-editorial-board-2024.html</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1399,7 +1403,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1409,12 +1413,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists 2024</t>
+          <t>A/P Rosa joins the Editorial Board of Discover Nano</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2024</t>
+          <t>discover-nano-editorial-board-2024</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1424,12 +1428,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2024.html</t>
+          <t>news/discover-nano-editorial-board-2024.html</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>top2pct-2024.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1440,11 +1444,6 @@
       <c r="J22" s="4" t="inlineStr">
         <is>
           <t>Done</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>4th consecutive year</t>
         </is>
       </c>
     </row>
@@ -1454,22 +1453,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>December 2024</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>A/P Rosa co-authors guidance on biocompatibility and dental-pulp regeneration</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists 2024</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>guidance-biocompat-pulp-2024</t>
+          <t>top2pct-scientists-2024</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1479,12 +1478,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>news/guidance-biocompat-pulp-2024.html</t>
+          <t>news/top2pct-scientists-2024.html</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>top2pct-2024.png</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1492,14 +1491,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>No hero image</t>
+          <t>4th consecutive year</t>
         </is>
       </c>
     </row>
@@ -1509,22 +1508,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>October 2024</t>
+          <t>December 2024</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed to the Board of Directors of the Academy of Dental Materials</t>
+          <t>A/P Rosa co-authors guidance on biocompatibility and dental-pulp regeneration</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>adm-board-member-2024</t>
+          <t>guidance-biocompat-pulp-2024</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1534,12 +1533,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>news/adm-board-member-2024.html</t>
+          <t>news/guidance-biocompat-pulp-2024.html</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>adm-board.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1547,14 +1546,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>CTA placeholder (#)</t>
+          <t>No hero image</t>
         </is>
       </c>
     </row>
@@ -1564,22 +1563,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 2024</t>
+          <t>October 2024</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Berita Harian features the NUCOHS Tooth Tissue Bank</t>
+          <t>A/P Rosa appointed to the Board of Directors of the Academy of Dental Materials</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>berita-harian-tooth-bank-2024</t>
+          <t>adm-board-member-2024</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1589,12 +1588,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>news/berita-harian-tooth-bank-2024.html</t>
+          <t>news/adm-board-member-2024.html</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>berita-harian-tooth-bank-2024.webp</t>
+          <t>adm-board.png</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1602,14 +1601,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>CTA placeholder (#)</t>
         </is>
       </c>
     </row>
@@ -1624,17 +1623,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>August 2024</t>
+          <t>September 2024</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Channel NewsAsia interviews A/P Rosa on the Tooth Tissue Bank</t>
+          <t>Berita Harian features the NUCOHS Tooth Tissue Bank</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>cna-tooth-bank-2024</t>
+          <t>berita-harian-tooth-bank-2024</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1644,12 +1643,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>news/cna-tooth-bank-2024.html</t>
+          <t>news/berita-harian-tooth-bank-2024.html</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>cna-tooth-bank-2024.jpg</t>
+          <t>berita-harian-tooth-bank-2024.webp</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1674,22 +1673,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Press</t>
+          <t>News</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>July 2024</t>
+          <t>August 2024</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The Straits Times: how Singapore's first Tooth Tissue Bank is advancing dental research</t>
+          <t>Channel NewsAsia interviews A/P Rosa on the Tooth Tissue Bank</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>straits-times-tooth-bank-2024</t>
+          <t>cna-tooth-bank-2024</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1699,12 +1698,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>news/straits-times-tooth-bank-2024.html</t>
+          <t>news/cna-tooth-bank-2024.html</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>cna-tooth-bank-2024.jpg</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1712,14 +1711,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>ST article screenshot (tooth-bank-st.png)</t>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -1729,22 +1728,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Press</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>March 2024</t>
+          <t>July 2024</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>A/P Rosa concludes his term as president of the IADR Dental Materials Group</t>
+          <t>The Straits Times: how Singapore's first Tooth Tissue Bank is advancing dental research</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>iadr-dmg-president-end-2024</t>
+          <t>straits-times-tooth-bank-2024</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1754,12 +1753,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>news/iadr-dmg-president-end-2024.html</t>
+          <t>news/straits-times-tooth-bank-2024.html</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>iadr-dmg-president-2024.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1767,14 +1766,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>ST article screenshot (tooth-bank-st.png)</t>
         </is>
       </c>
     </row>
@@ -1784,22 +1783,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>March 2024</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Clarice Sabino wins the 2023 IADR Kulzer Travel Award</t>
+          <t>A/P Rosa concludes his term as president of the IADR Dental Materials Group</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>iadr-kulzer-travel-award-clarice-sabino-2023</t>
+          <t>iadr-dmg-president-end-2024</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1809,12 +1808,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>news/iadr-kulzer-travel-award-clarice-sabino-2023.html</t>
+          <t>news/iadr-dmg-president-end-2024.html</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>iadr-kulzer-award-clarice-sabino-2023.jpg</t>
+          <t>iadr-dmg-president-2024.png</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1822,9 +1821,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1848,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Priti Pragati Rath receives the IADR Kulzer Award 2023</t>
+          <t>Clarice Sabino wins the 2023 IADR Kulzer Travel Award</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>iadr-kulzer-award-priti-pragati-rath-2023</t>
+          <t>iadr-kulzer-travel-award-clarice-sabino-2023</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1859,12 +1863,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>news/iadr-kulzer-award-priti-pragati-rath-2023.html</t>
+          <t>news/iadr-kulzer-travel-award-clarice-sabino-2023.html</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>iadr-kulzer-award-priti-pragati-rath.jpg</t>
+          <t>iadr-kulzer-award-clarice-sabino-2023.jpg</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1875,11 +1879,6 @@
       <c r="J30" s="4" t="inlineStr">
         <is>
           <t>Done</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Supervisor: A/P Rosa</t>
         </is>
       </c>
     </row>
@@ -1894,17 +1893,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>November 2023</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A/P Rosa's work selected for the JDR Editor's Choice Collection 2023</t>
+          <t>Priti Pragati Rath receives the IADR Kulzer Award 2023</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>jdr-editors-choice-collection-2023</t>
+          <t>iadr-kulzer-award-priti-pragati-rath-2023</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1914,12 +1913,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>news/jdr-editors-choice-collection-2023.html</t>
+          <t>news/iadr-kulzer-award-priti-pragati-rath-2023.html</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>jdr-editor-choice-2023.png</t>
+          <t>iadr-kulzer-award-priti-pragati-rath.jpg</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1930,6 +1929,11 @@
       <c r="J31" s="4" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Supervisor: A/P Rosa</t>
         </is>
       </c>
     </row>
@@ -1944,17 +1948,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>October 2023</t>
+          <t>November 2023</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>A/P Rosa becomes a Fellow of the Academy of Dental Materials</t>
+          <t>A/P Rosa's work selected for the JDR Editor's Choice Collection 2023</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>adm-fellow-2023</t>
+          <t>jdr-editors-choice-collection-2023</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1964,12 +1968,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>news/adm-fellow-2023.html</t>
+          <t>news/jdr-editors-choice-collection-2023.html</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>jdr-editor-choice-2023.png</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1977,14 +1981,9 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>No hero image</t>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2004,12 +2003,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>A/P Rosa recognised in the World's Top 2% most-cited scientists 2023</t>
+          <t>A/P Rosa becomes a Fellow of the Academy of Dental Materials</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2023</t>
+          <t>adm-fellow-2023</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2019,12 +2018,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2023.html</t>
+          <t>news/adm-fellow-2023.html</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>top2pct-2023.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2032,14 +2031,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="J33" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>3rd consecutive year</t>
+          <t>No hero image</t>
         </is>
       </c>
     </row>
@@ -2054,17 +2053,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>April 2023</t>
+          <t>October 2023</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>UFPEL and NUS win One Health research grants</t>
+          <t>A/P Rosa recognised in the World's Top 2% most-cited scientists 2023</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ufpel-nus-one-health-2023</t>
+          <t>top2pct-scientists-2023</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2074,12 +2073,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>news/ufpel-nus-one-health-2023.html</t>
+          <t>news/top2pct-scientists-2023.html</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>ufpel-nus-research-collaboration.png</t>
+          <t>top2pct-2023.png</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2087,14 +2086,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>3rd consecutive year</t>
         </is>
       </c>
     </row>
@@ -2109,17 +2108,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>October 2022</t>
+          <t>April 2023</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A/P Rosa among the World's Top 2% most-cited scientists (2nd consecutive year)</t>
+          <t>UFPEL and NUS win One Health research grants</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2022</t>
+          <t>ufpel-nus-one-health-2023</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2129,12 +2128,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2022.html</t>
+          <t>news/ufpel-nus-one-health-2023.html</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>top2pct-2022.png</t>
+          <t>ufpel-nus-research-collaboration.png</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2142,14 +2141,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2nd consecutive year</t>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -2164,17 +2163,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>October 2022</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Melissa Koh receives the IADR Pediatric Oral Health Research Group Student Award 2021</t>
+          <t>A/P Rosa among the World's Top 2% most-cited scientists (2nd consecutive year)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>iadr-pediatric-award-melissa-koh-2021</t>
+          <t>top2pct-scientists-2022</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2184,12 +2183,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>news/iadr-pediatric-award-melissa-koh-2021.html</t>
+          <t>news/top2pct-scientists-2022.html</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>top2pct-2022.png</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2204,7 +2203,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Supervisor: A/P Rosa</t>
+          <t>2nd consecutive year</t>
         </is>
       </c>
     </row>
@@ -2219,17 +2218,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>July 2021</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>A/P Rosa receives the 2021 IADR Stephen Bayne Mid-Career Award</t>
+          <t>Melissa Koh receives the IADR Pediatric Oral Health Research Group Student Award 2021</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>iadr-bayne-midcareer-2021</t>
+          <t>iadr-pediatric-award-melissa-koh-2021</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2239,12 +2238,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>news/iadr-bayne-midcareer-award-2021.html</t>
+          <t>news/iadr-pediatric-award-melissa-koh-2021.html</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>iadr-bayne-midcareer-award-2021.jpg</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2252,14 +2251,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J37" s="6" t="inlineStr">
+      <c r="J37" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>Supervisor: A/P Rosa</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2278,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A/P Rosa receives the IADR Distinguished Young Investigator Award</t>
+          <t>A/P Rosa receives the 2021 IADR Stephen Bayne Mid-Career Award</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>iadr-young-investigator-2021</t>
+          <t>iadr-bayne-midcareer-2021</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2294,12 +2293,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>news/iadr-young-investigator-award-2021.html</t>
+          <t>news/iadr-bayne-midcareer-award-2021.html</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>iadr-young-investigator-award-2021.webp</t>
+          <t>iadr-bayne-midcareer-award-2021.jpg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2334,12 +2333,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Four NUS Dentistry researchers in the World's Top 2% most-cited scientists</t>
+          <t>A/P Rosa receives the IADR Distinguished Young Investigator Award</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>top2pct-scientists-2021</t>
+          <t>iadr-young-investigator-2021</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2349,12 +2348,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>news/top2pct-scientists-2021.html</t>
+          <t>news/iadr-young-investigator-award-2021.html</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>top2pct-2021.png</t>
+          <t>iadr-young-investigator-award-2021.webp</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2362,14 +2361,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>One of four NUS Dentistry researchers that year</t>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -2384,17 +2383,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>June 2021</t>
+          <t>July 2021</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Best graphical abstract — eCells &amp; Materials</t>
+          <t>Four NUS Dentistry researchers in the World's Top 2% most-cited scientists</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ecm-graphical-abstract-2021</t>
+          <t>top2pct-scientists-2021</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2404,12 +2403,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>news/ecm-graphical-abstract-2021.html</t>
+          <t>news/top2pct-scientists-2021.html</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>ecm-graphical-abstract-2021.jpg</t>
+          <t>top2pct-2021.png</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2417,14 +2416,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="J40" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Ultra-wide 858×229; contain mode</t>
+          <t>One of four NUS Dentistry researchers that year</t>
         </is>
       </c>
     </row>
@@ -2434,22 +2433,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>June 2021</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of Dental Materials</t>
+          <t>Best graphical abstract — eCells &amp; Materials</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>dental-materials-editorial-board-2020</t>
+          <t>ecm-graphical-abstract-2021</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2459,12 +2458,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>news/dental-materials-editorial-board-2020.html</t>
+          <t>news/ecm-graphical-abstract-2021.html</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ecm-graphical-abstract-2021.jpg</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2472,14 +2471,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr">
+      <c r="J41" s="6" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>No hero image (had a mismatched RSC Sustainability cover wired in by mistake, removed 2026-08-04)</t>
+          <t>Ultra-wide 858×229; contain mode</t>
         </is>
       </c>
     </row>
@@ -2499,12 +2498,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of JADA FS</t>
+          <t>A/P Rosa joins the Editorial Board of Dental Materials</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>jada-fs-editorial-board-2020</t>
+          <t>dental-materials-editorial-board-2020</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2514,7 +2513,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>news/jada-fs-editorial-board-2020.html</t>
+          <t>news/dental-materials-editorial-board-2020.html</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2530,6 +2529,11 @@
       <c r="J42" s="4" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>No hero image (had a mismatched RSC Sustainability cover wired in by mistake, removed 2026-08-04)</t>
         </is>
       </c>
     </row>
@@ -2549,12 +2553,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed Associate Editor of the Journal of Prosthodontics</t>
+          <t>A/P Rosa joins the Editorial Board of JADA FS</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>journal-prosthodontics-associate-editor-2020</t>
+          <t>jada-fs-editorial-board-2020</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2564,7 +2568,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>news/journal-prosthodontics-associate-editor-2020.html</t>
+          <t>news/jada-fs-editorial-board-2020.html</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2589,22 +2593,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Institutional</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>December 2020</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Dental DART — protective tent for safer dentistry during the pandemic</t>
+          <t>A/P Rosa appointed Associate Editor of the Journal of Prosthodontics</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>dental-dart-aerosol-2020</t>
+          <t>journal-prosthodontics-associate-editor-2020</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2614,12 +2618,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>news/dental-dart-aerosol-2020.html</t>
+          <t>news/journal-prosthodontics-associate-editor-2020.html</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>dental-dart-01…04.jpg</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2630,11 +2634,6 @@
       <c r="J44" s="4" t="inlineStr">
         <is>
           <t>Done</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>COVID-era aerosol shield; 4 photos</t>
         </is>
       </c>
     </row>
@@ -2644,22 +2643,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Institutional</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>February 2020</t>
+          <t>December 2020</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Two papers among the 25 most-cited in Dental Materials</t>
+          <t>Dental DART — protective tent for safer dentistry during the pandemic</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>dental-materials-top25-2020</t>
+          <t>dental-dart-aerosol-2020</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2669,12 +2668,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>news/dental-materials-top25-2020.html</t>
+          <t>news/dental-dart-aerosol-2020.html</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>dental-materials-top25-2020.png</t>
+          <t>dental-dart-01…04.jpg</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2682,14 +2681,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="J45" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Needs asset; text in PDFs</t>
+          <t>COVID-era aerosol shield; 4 photos</t>
         </is>
       </c>
     </row>
@@ -2699,22 +2698,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>February 2020</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Scientific Advisory Board of the Journal of Endodontics</t>
+          <t>Two papers among the 25 most-cited in Dental Materials</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>joe-scientific-advisory-board-2019</t>
+          <t>dental-materials-top25-2020</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2724,12 +2723,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>news/joe-scientific-advisory-board-2019.html</t>
+          <t>news/dental-materials-top25-2020.html</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>dental-materials-top25-2020.png</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2737,9 +2736,14 @@
           <t>EN/ES/PT/FR/中文</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Needs asset; text in PDFs</t>
         </is>
       </c>
     </row>
@@ -2759,12 +2763,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>A/P Rosa appointed Associate Editor of Emergent Materials</t>
+          <t>A/P Rosa joins the Scientific Advisory Board of the Journal of Endodontics</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>emergent-materials-associate-editor-2019</t>
+          <t>joe-scientific-advisory-board-2019</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2774,7 +2778,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>news/emergent-materials-associate-editor-2019.html</t>
+          <t>news/joe-scientific-advisory-board-2019.html</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2799,22 +2803,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Appointment</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Klara Koh receives the IADR-SEA Hatton Award Junior Category 2018</t>
+          <t>A/P Rosa appointed Associate Editor of Emergent Materials</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>iadr-sea-hatton-junior-klara-koh-2018</t>
+          <t>emergent-materials-associate-editor-2019</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2824,7 +2828,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>news/iadr-sea-hatton-junior-klara-koh-2018.html</t>
+          <t>news/emergent-materials-associate-editor-2019.html</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2840,11 +2844,6 @@
       <c r="J48" s="4" t="inlineStr">
         <is>
           <t>Done</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Supervisor: A/P Rosa</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2853,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Appointment</t>
+          <t>Award</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2864,12 +2863,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>A/P Rosa joins the Editorial Board of the Journal of Dental Research</t>
+          <t>Klara Koh receives the IADR-SEA Hatton Award Junior Category 2018</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>jdr-editorial-board-2018</t>
+          <t>iadr-sea-hatton-junior-klara-koh-2018</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2879,7 +2878,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>news/jdr-editorial-board-2018.html</t>
+          <t>news/iadr-sea-hatton-junior-klara-koh-2018.html</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2899,7 +2898,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>No hero image (had the jdr-editors-choice-collection-2023 paper card wired in by mistake, removed 2026-08-04)</t>
+          <t>Supervisor: A/P Rosa</t>
         </is>
       </c>
     </row>
@@ -2909,50 +2908,105 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>Appointment</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>A/P Rosa joins the Editorial Board of the Journal of Dental Research</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>jdr-editorial-board-2018</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>news/jdr-editorial-board-2018.html</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>EN/ES/PT/FR/中文</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>No hero image (had the jdr-editors-choice-collection-2023 paper card wired in by mistake, removed 2026-08-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>45</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>Award</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>November 2018</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Two of A/P Rosa's papers among the 100 most-cited in regenerative endodontics</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>two-top-cited-papers-regenerative-endodontics-2018</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
         <is>
           <t>news/two-top-cited-papers-regenerative-endodontics-2018.html</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>two-top-cited-regenerative-endodontics.png</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>EN/ES/PT/FR/中文</t>
-        </is>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>EN/ES/PT/FR/中文</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t>#26 JDR 2013 / #98 Int Dent J 2011 per JOE 2018 bibliometric analysis</t>
         </is>

</xml_diff>